<commit_message>
Lexical quality filter: Southern orthography, rare glosses, corpus attestation and beginner core set; updated evaluation
</commit_message>
<xml_diff>
--- a/experimentos/lre/revision/hoja-aimara.xlsx
+++ b/experimentos/lre/revision/hoja-aimara.xlsx
@@ -474,17 +474,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>A001</t>
+          <t>AN001</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>ñuñu</t>
+          <t>apjaña</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>mama, teta, seno, pecho</t>
+          <t>separar, apartar</t>
         </is>
       </c>
       <c r="D2" s="2" t="n"/>
@@ -494,17 +494,17 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>A002</t>
+          <t>AN002</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>ch'uxña</t>
+          <t>jachaña</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>inmaduro, no maduro, verde</t>
+          <t>llorar</t>
         </is>
       </c>
       <c r="D3" s="2" t="n"/>
@@ -514,17 +514,17 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>A003</t>
+          <t>AN003</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>jutaña</t>
+          <t>mujlli</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>venir</t>
+          <t>codo</t>
         </is>
       </c>
       <c r="D4" s="2" t="n"/>
@@ -534,17 +534,17 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>A004</t>
+          <t>AN004</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>ch'amuña</t>
+          <t>paqallqu</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>chupar</t>
+          <t>siete</t>
         </is>
       </c>
       <c r="D5" s="2" t="n"/>
@@ -554,17 +554,17 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>A005</t>
+          <t>AN005</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>siqi</t>
+          <t>thikhiña</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>línea</t>
+          <t>mezclar, mixturar</t>
         </is>
       </c>
       <c r="D6" s="2" t="n"/>
@@ -574,17 +574,17 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>A006</t>
+          <t>AN006</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>anu</t>
+          <t>phisna</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>perro</t>
+          <t>liviano</t>
         </is>
       </c>
       <c r="D7" s="2" t="n"/>
@@ -594,17 +594,17 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>A007</t>
+          <t>AN007</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>manq'aña</t>
+          <t>qura</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>comer</t>
+          <t>hierba, pasto</t>
         </is>
       </c>
       <c r="D8" s="2" t="n"/>
@@ -614,17 +614,17 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>A008</t>
+          <t>AN008</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>achichi</t>
+          <t>ch'iyara</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>viejo, anciano</t>
+          <t>negro</t>
         </is>
       </c>
       <c r="D9" s="2" t="n"/>
@@ -634,17 +634,17 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>A009</t>
+          <t>AN009</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>samaña</t>
+          <t>tunka paqallquni</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>descansar, reposar</t>
+          <t>diecisiete</t>
         </is>
       </c>
       <c r="D10" s="2" t="n"/>
@@ -654,17 +654,17 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>A010</t>
+          <t>AN010</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>wayna</t>
+          <t>uta pata</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>hombre joven, mozo, muchacho</t>
+          <t>tejado</t>
         </is>
       </c>
       <c r="D11" s="2" t="n"/>
@@ -674,17 +674,17 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>A011</t>
+          <t>AN011</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>iñu</t>
+          <t>jiwaqayaña</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>huérfano/ huérfana</t>
+          <t>apagar</t>
         </is>
       </c>
       <c r="D12" s="2" t="n"/>
@@ -694,17 +694,17 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>A012</t>
+          <t>AN012</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>apaña</t>
+          <t>imilla wawa</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>llevar en la mano</t>
+          <t>hija</t>
         </is>
       </c>
       <c r="D13" s="2" t="n"/>
@@ -714,17 +714,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>A013</t>
+          <t>AN013</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>nina</t>
+          <t>qinaya</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>fuego</t>
+          <t>nube</t>
         </is>
       </c>
       <c r="D14" s="2" t="n"/>
@@ -734,17 +734,17 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>A014</t>
+          <t>AN014</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>phisna</t>
+          <t>wayra</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>liviano</t>
+          <t>viento</t>
         </is>
       </c>
       <c r="D15" s="2" t="n"/>
@@ -754,17 +754,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>A015</t>
+          <t>AN015</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>urqu</t>
+          <t>tawaqu</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>macho</t>
+          <t>señorita</t>
         </is>
       </c>
       <c r="D16" s="2" t="n"/>
@@ -774,17 +774,17 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>A016</t>
+          <t>AN016</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>kupi</t>
+          <t>panqara</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>derecha</t>
+          <t>flor</t>
         </is>
       </c>
       <c r="D17" s="2" t="n"/>
@@ -794,17 +794,17 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>A017</t>
+          <t>AN017</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>inti</t>
+          <t>jutaña</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>sol</t>
+          <t>venir</t>
         </is>
       </c>
       <c r="D18" s="2" t="n"/>
@@ -814,17 +814,17 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>A018</t>
+          <t>AN018</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>yäqaña</t>
+          <t>wiphala</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>dignidad</t>
+          <t>bandera</t>
         </is>
       </c>
       <c r="D19" s="2" t="n"/>
@@ -834,17 +834,17 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>A019</t>
+          <t>AN019</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>pataka</t>
+          <t>sich'i</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>ciento, cien</t>
+          <t>línea</t>
         </is>
       </c>
       <c r="D20" s="2" t="n"/>
@@ -854,17 +854,17 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>A020</t>
+          <t>AN020</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>jukumari</t>
+          <t>lurañ yänaka</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>oso de anteojos</t>
+          <t>tecnología, técnica</t>
         </is>
       </c>
       <c r="D21" s="2" t="n"/>
@@ -874,17 +874,17 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>A021</t>
+          <t>AN021</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>jila</t>
+          <t>nasa</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>hermano</t>
+          <t>nariz</t>
         </is>
       </c>
       <c r="D22" s="2" t="n"/>
@@ -894,17 +894,17 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>A022</t>
+          <t>AN022</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>saxra</t>
+          <t>wallqanqa</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>viento, ventisca, ventarrón</t>
+          <t>escudo de armas, escudo, armas</t>
         </is>
       </c>
       <c r="D23" s="2" t="n"/>
@@ -914,17 +914,17 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>A023</t>
+          <t>AN023</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>imaña</t>
+          <t>jaljaña</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>conservar, retener</t>
+          <t>dividir</t>
         </is>
       </c>
       <c r="D24" s="2" t="n"/>
@@ -934,17 +934,17 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>A024</t>
+          <t>AN024</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>laxra chinja</t>
+          <t>puquta</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>trabalenguas</t>
+          <t>banana, banano, cambur</t>
         </is>
       </c>
       <c r="D25" s="2" t="n"/>
@@ -954,17 +954,17 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>A025</t>
+          <t>AN025</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>nayra</t>
+          <t>qamaqi</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>ojo</t>
+          <t>zorro</t>
         </is>
       </c>
       <c r="D26" s="2" t="n"/>
@@ -974,17 +974,17 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>A026</t>
+          <t>AN026</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>asxaraña</t>
+          <t>arumita</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>temer, tener miedo</t>
+          <t>naranja</t>
         </is>
       </c>
       <c r="D27" s="2" t="n"/>
@@ -994,17 +994,17 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>A027</t>
+          <t>AN027</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>thaya</t>
+          <t>achachi</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>viento</t>
+          <t>viejo</t>
         </is>
       </c>
       <c r="D28" s="2" t="n"/>
@@ -1014,17 +1014,17 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>A028</t>
+          <t>AN028</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>chacha</t>
+          <t>jatha</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>marido, esposo</t>
+          <t>semilla</t>
         </is>
       </c>
       <c r="D29" s="2" t="n"/>
@@ -1034,17 +1034,17 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>A029</t>
+          <t>AN029</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>lap'a</t>
+          <t>q'illu</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>piojo</t>
+          <t>amarillo</t>
         </is>
       </c>
       <c r="D30" s="2" t="n"/>
@@ -1054,7 +1054,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>A030</t>
+          <t>AN030</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1074,17 +1074,17 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>A031</t>
+          <t>AN031</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>paqallqu</t>
+          <t>achichi</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>siete</t>
+          <t>viejo, anciano</t>
         </is>
       </c>
       <c r="D32" s="2" t="n"/>
@@ -1094,17 +1094,17 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>A032</t>
+          <t>AN032</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>achachi</t>
+          <t>ch'amuña</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>viejo</t>
+          <t>chupar</t>
         </is>
       </c>
       <c r="D33" s="2" t="n"/>
@@ -1114,17 +1114,17 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>A033</t>
+          <t>AN033</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>wich'inkha</t>
+          <t>anu</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>cola</t>
+          <t>perro</t>
         </is>
       </c>
       <c r="D34" s="2" t="n"/>
@@ -1134,17 +1134,17 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>A034</t>
+          <t>AN034</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>saphi</t>
+          <t>chhiqha</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>raíz</t>
+          <t>ala</t>
         </is>
       </c>
       <c r="D35" s="2" t="n"/>
@@ -1154,17 +1154,17 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>A035</t>
+          <t>AN035</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>chika aruma</t>
+          <t>jiwq'i</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>medianoche</t>
+          <t>humo, jumo</t>
         </is>
       </c>
       <c r="D36" s="2" t="n"/>
@@ -1174,17 +1174,17 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>A036</t>
+          <t>AN036</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>nukhuña</t>
+          <t>waña</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>empujar</t>
+          <t>seco</t>
         </is>
       </c>
       <c r="D37" s="2" t="n"/>
@@ -1194,17 +1194,17 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>A037</t>
+          <t>AN037</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>aka</t>
+          <t>chara</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>esto, este, esta</t>
+          <t>pierna</t>
         </is>
       </c>
       <c r="D38" s="2" t="n"/>
@@ -1214,17 +1214,17 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>A038</t>
+          <t>AN038</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>ch'alla</t>
+          <t>phisqa</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>arena</t>
+          <t>cinco</t>
         </is>
       </c>
       <c r="D39" s="2" t="n"/>
@@ -1234,17 +1234,17 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>A039</t>
+          <t>AN039</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>jaqi</t>
+          <t>aycha</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>ser humano</t>
+          <t>carne</t>
         </is>
       </c>
       <c r="D40" s="2" t="n"/>
@@ -1254,17 +1254,17 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>A040</t>
+          <t>AN040</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>phaxsi uru</t>
+          <t>chikata</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>lunes</t>
+          <t>mitad</t>
         </is>
       </c>
       <c r="D41" s="2" t="n"/>
@@ -1274,17 +1274,17 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>A041</t>
+          <t>AN041</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>jinchu</t>
+          <t>llink'i laq'a</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>{{t+|es|oreja|f}, oído</t>
+          <t>arcilla, barro, argilla</t>
         </is>
       </c>
       <c r="D42" s="2" t="n"/>
@@ -1294,17 +1294,17 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>A042</t>
+          <t>AN042</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>kayu</t>
+          <t>p'iqi</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>pie</t>
+          <t>cabeza</t>
         </is>
       </c>
       <c r="D43" s="2" t="n"/>
@@ -1314,17 +1314,17 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>A043</t>
+          <t>AN043</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>achikt'aña</t>
+          <t>airu</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>rogarse, implorar</t>
+          <t>planta</t>
         </is>
       </c>
       <c r="D44" s="2" t="n"/>
@@ -1334,17 +1334,17 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>A044</t>
+          <t>AN044</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>atiniña</t>
+          <t>wank'u</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>libertad</t>
+          <t>conejo</t>
         </is>
       </c>
       <c r="D45" s="2" t="n"/>
@@ -1354,17 +1354,17 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>A045</t>
+          <t>AN045</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>machaqa</t>
+          <t>awkinaka</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>nuevo</t>
+          <t>padres</t>
         </is>
       </c>
       <c r="D46" s="2" t="n"/>
@@ -1374,17 +1374,17 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>A046</t>
+          <t>AN046</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>achuqalla</t>
+          <t>akapacha</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>comadreja</t>
+          <t>este mundo</t>
         </is>
       </c>
       <c r="D47" s="2" t="n"/>
@@ -1394,17 +1394,17 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>A047</t>
+          <t>AN047</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>uma</t>
+          <t>atiniña</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>agua líquida</t>
+          <t>libertad</t>
         </is>
       </c>
       <c r="D48" s="2" t="n"/>
@@ -1414,17 +1414,17 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>A048</t>
+          <t>AN048</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>tuyuña</t>
+          <t>churaña</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>nadar</t>
+          <t>dar</t>
         </is>
       </c>
       <c r="D49" s="2" t="n"/>
@@ -1434,17 +1434,17 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>A049</t>
+          <t>AN049</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>ch'iyara</t>
+          <t>saphi</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>negro</t>
+          <t>raíz</t>
         </is>
       </c>
       <c r="D50" s="2" t="n"/>
@@ -1454,17 +1454,17 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>A050</t>
+          <t>AN050</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>umata awtjaaña</t>
+          <t>arumanthi</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>sed</t>
+          <t>madrugada, mañana, antelucano</t>
         </is>
       </c>
       <c r="D51" s="2" t="n"/>
@@ -1474,17 +1474,17 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>A051</t>
+          <t>AN051</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>munaña</t>
+          <t>qhuyphi</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>querer</t>
+          <t>alta (voz), ruidoso</t>
         </is>
       </c>
       <c r="D52" s="2" t="n"/>
@@ -1494,17 +1494,17 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>A052</t>
+          <t>AN052</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>ch'usa</t>
+          <t>ispillu</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>vacío</t>
+          <t>labio</t>
         </is>
       </c>
       <c r="D53" s="2" t="n"/>
@@ -1514,17 +1514,17 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>A053</t>
+          <t>AN053</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>waxra</t>
+          <t>alaya</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>cuerno</t>
+          <t>arriba</t>
         </is>
       </c>
       <c r="D54" s="2" t="n"/>
@@ -1534,17 +1534,17 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>A054</t>
+          <t>AN054</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>ch'iwi</t>
+          <t>wich'inkha</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>sombra</t>
+          <t>cola</t>
         </is>
       </c>
       <c r="D55" s="2" t="n"/>
@@ -1554,17 +1554,17 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>A055</t>
+          <t>AN055</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>añuthaya</t>
+          <t>chika aruma</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>zorro hediondo, zorrillo, zorrino</t>
+          <t>medianoche</t>
         </is>
       </c>
       <c r="D56" s="2" t="n"/>
@@ -1574,17 +1574,17 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>A056</t>
+          <t>AN056</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>t'ant'a</t>
+          <t>ñuñu</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>pan</t>
+          <t>mama, teta, seno, pecho</t>
         </is>
       </c>
       <c r="D57" s="2" t="n"/>
@@ -1594,17 +1594,17 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>A057</t>
+          <t>AN057</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>aqu</t>
+          <t>chupika</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>arena</t>
+          <t>rojo</t>
         </is>
       </c>
       <c r="D58" s="2" t="n"/>
@@ -1614,17 +1614,17 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>A058</t>
+          <t>AN058</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>ch'ankha</t>
+          <t>jalanta</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>hilo</t>
+          <t>oeste, poniente</t>
         </is>
       </c>
       <c r="D59" s="2" t="n"/>
@@ -1634,17 +1634,17 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>A059</t>
+          <t>AN059</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>chara</t>
+          <t>tuyuña</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>pierna</t>
+          <t>nadar</t>
         </is>
       </c>
       <c r="D60" s="2" t="n"/>
@@ -1654,17 +1654,17 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>A060</t>
+          <t>AN060</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>imantaña</t>
+          <t>jiwaña</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>esconder</t>
+          <t>morir, muerto</t>
         </is>
       </c>
       <c r="D61" s="2" t="n"/>
@@ -1674,17 +1674,17 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>A061</t>
+          <t>AN061</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>chupika</t>
+          <t>jiq'i</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>rojo</t>
+          <t>humo</t>
         </is>
       </c>
       <c r="D62" s="2" t="n"/>
@@ -1694,17 +1694,17 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>A062</t>
+          <t>AN062</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>marmi</t>
+          <t>challwa</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>único</t>
+          <t>pescado</t>
         </is>
       </c>
       <c r="D63" s="2" t="n"/>
@@ -1714,17 +1714,17 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>A063</t>
+          <t>AN063</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>jiq'i</t>
+          <t>kimsaqallqu</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>humo</t>
+          <t>ocho</t>
         </is>
       </c>
       <c r="D64" s="2" t="n"/>
@@ -1734,17 +1734,17 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>A064</t>
+          <t>AN064</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>wila</t>
+          <t>inti</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>rojo</t>
+          <t>sol</t>
         </is>
       </c>
       <c r="D65" s="2" t="n"/>
@@ -1754,17 +1754,17 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>A065</t>
+          <t>AN065</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>jamach'i</t>
+          <t>kayu</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>pájaro</t>
+          <t>pie</t>
         </is>
       </c>
       <c r="D66" s="2" t="n"/>
@@ -1774,17 +1774,17 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>A066</t>
+          <t>AN066</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>juma</t>
+          <t>ch'akha</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>usted, tú, vos</t>
+          <t>hueso</t>
         </is>
       </c>
       <c r="D67" s="2" t="n"/>
@@ -1794,17 +1794,17 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>A067</t>
+          <t>AN067</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>phisqa</t>
+          <t>wila</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>cinco</t>
+          <t>rojo</t>
         </is>
       </c>
       <c r="D68" s="2" t="n"/>
@@ -1814,17 +1814,17 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>A068</t>
+          <t>AN068</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>jaqi</t>
+          <t>laphi</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>persona</t>
+          <t>hoja</t>
         </is>
       </c>
       <c r="D69" s="2" t="n"/>
@@ -1834,17 +1834,17 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>A069</t>
+          <t>AN069</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>k'awna q'illu</t>
+          <t>mistuña</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>yema (de huevo)</t>
+          <t>salir</t>
         </is>
       </c>
       <c r="D70" s="2" t="n"/>
@@ -1854,17 +1854,17 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>A070</t>
+          <t>AN070</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>jallq'aña</t>
+          <t>liq'iña</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>lamer</t>
+          <t>golpear</t>
         </is>
       </c>
       <c r="D71" s="2" t="n"/>
@@ -1874,17 +1874,17 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>A071</t>
+          <t>AN071</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>chhiqha</t>
+          <t>jathi</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>ala</t>
+          <t>pesado</t>
         </is>
       </c>
       <c r="D72" s="2" t="n"/>
@@ -1894,17 +1894,17 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>A072</t>
+          <t>AN072</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>q'itha</t>
+          <t>chupila</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>esperma</t>
+          <t>vagina</t>
         </is>
       </c>
       <c r="D73" s="2" t="n"/>
@@ -1914,17 +1914,17 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>A073</t>
+          <t>AN073</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>t'arwa</t>
+          <t>usuchaña</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>lana</t>
+          <t>dañar, herir</t>
         </is>
       </c>
       <c r="D74" s="2" t="n"/>
@@ -1934,17 +1934,17 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>A074</t>
+          <t>AN074</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>k'umara</t>
+          <t>qhatu</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>sano, salud</t>
+          <t>mercado</t>
         </is>
       </c>
       <c r="D75" s="2" t="n"/>
@@ -1954,17 +1954,17 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>A075</t>
+          <t>AN075</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>qhilla</t>
+          <t>uru</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>ceniza</t>
+          <t>día</t>
         </is>
       </c>
       <c r="D76" s="2" t="n"/>
@@ -1974,17 +1974,17 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>A076</t>
+          <t>AN076</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>aruma</t>
+          <t>jila</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>noche</t>
+          <t>hermano</t>
         </is>
       </c>
       <c r="D77" s="2" t="n"/>
@@ -1994,17 +1994,17 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>A077</t>
+          <t>AN077</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>maysarnukuta</t>
+          <t>q'uchu</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>descuidado, irresponsable, negligente</t>
+          <t>canción, rola</t>
         </is>
       </c>
       <c r="D78" s="2" t="n"/>
@@ -2014,17 +2014,17 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>A078</t>
+          <t>AN078</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>wayra</t>
+          <t>imantaña</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>viento</t>
+          <t>esconder</t>
         </is>
       </c>
       <c r="D79" s="2" t="n"/>
@@ -2034,17 +2034,17 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>A079</t>
+          <t>AN079</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>qura</t>
+          <t>yatiña</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>hierba, pasto</t>
+          <t>saber</t>
         </is>
       </c>
       <c r="D80" s="2" t="n"/>
@@ -2054,17 +2054,17 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>A080</t>
+          <t>AN080</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>jila</t>
+          <t>lluqu</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>hermano/hermana</t>
+          <t>corazón</t>
         </is>
       </c>
       <c r="D81" s="2" t="n"/>
@@ -2074,17 +2074,17 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>A081</t>
+          <t>AN081</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>sarnaqaña uñtapa</t>
+          <t>uraqita</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>orientación sexual</t>
+          <t>geografía</t>
         </is>
       </c>
       <c r="D82" s="2" t="n"/>
@@ -2094,17 +2094,17 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>A082</t>
+          <t>AN082</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>sillu</t>
+          <t>warmi</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>uña</t>
+          <t>mujer</t>
         </is>
       </c>
       <c r="D83" s="2" t="n"/>
@@ -2114,17 +2114,17 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>A083</t>
+          <t>AN083</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>alaya</t>
+          <t>jawira</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>arriba</t>
+          <t>río</t>
         </is>
       </c>
       <c r="D84" s="2" t="n"/>
@@ -2134,17 +2134,17 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>A084</t>
+          <t>AN084</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>ist'aña</t>
+          <t>laruña</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>oír</t>
+          <t>reír</t>
         </is>
       </c>
       <c r="D85" s="2" t="n"/>
@@ -2154,17 +2154,17 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>A085</t>
+          <t>AN085</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>jariña</t>
+          <t>llätunka</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>lavar</t>
+          <t>nueve</t>
         </is>
       </c>
       <c r="D86" s="2" t="n"/>
@@ -2174,17 +2174,17 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>A086</t>
+          <t>AN086</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>qanlli</t>
+          <t>tunka kimsani</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>hormiga, huasho, shishi</t>
+          <t>trece</t>
         </is>
       </c>
       <c r="D87" s="2" t="n"/>
@@ -2194,17 +2194,17 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>A087</t>
+          <t>AN087</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>jisk'a</t>
+          <t>jamach'i</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>pequeño, chico, parvo</t>
+          <t>pájaro</t>
         </is>
       </c>
       <c r="D88" s="2" t="n"/>
@@ -2214,17 +2214,17 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>A088</t>
+          <t>AN088</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>q'illu</t>
+          <t>quqa</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>amarillo</t>
+          <t>árbol</t>
         </is>
       </c>
       <c r="D89" s="2" t="n"/>
@@ -2234,17 +2234,17 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>A089</t>
+          <t>AN089</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>jiwaña</t>
+          <t>manq'aña</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>morir, muerto</t>
+          <t>comer</t>
         </is>
       </c>
       <c r="D90" s="2" t="n"/>
@@ -2254,17 +2254,17 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>A090</t>
+          <t>AN090</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>kimsaqallqu</t>
+          <t>ch'alla</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>ocho</t>
+          <t>arena</t>
         </is>
       </c>
       <c r="D91" s="2" t="n"/>
@@ -2274,17 +2274,17 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>A091</t>
+          <t>AN091</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>mujlli</t>
+          <t>waxra</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>codo</t>
+          <t>cuerno</t>
         </is>
       </c>
       <c r="D92" s="2" t="n"/>
@@ -2294,17 +2294,17 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>A092</t>
+          <t>AN092</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>tayiksuyu</t>
+          <t>yatxatawi</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>tayikistán</t>
+          <t>ciencia</t>
         </is>
       </c>
       <c r="D93" s="2" t="n"/>
@@ -2314,17 +2314,17 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>A093</t>
+          <t>AN093</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>llätunka</t>
+          <t>jaqi</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>nueve</t>
+          <t>persona</t>
         </is>
       </c>
       <c r="D94" s="2" t="n"/>
@@ -2334,17 +2334,17 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>A094</t>
+          <t>AN094</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>wasuru</t>
+          <t>tikitiki</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>ayer</t>
+          <t>gallina de agua</t>
         </is>
       </c>
       <c r="D95" s="2" t="n"/>
@@ -2354,17 +2354,17 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>A095</t>
+          <t>AN095</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>warmi</t>
+          <t>machaqa</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>mujer</t>
+          <t>nuevo</t>
         </is>
       </c>
       <c r="D96" s="2" t="n"/>
@@ -2374,17 +2374,17 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>A096</t>
+          <t>AN096</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>ajllita</t>
+          <t>allu</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>escogido, elegido</t>
+          <t>pene</t>
         </is>
       </c>
       <c r="D97" s="2" t="n"/>
@@ -2394,17 +2394,17 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>A097</t>
+          <t>AN097</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>chhaqachhaqa</t>
+          <t>jan wali</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>horizonte</t>
+          <t>peligroso, brígido, fortunal</t>
         </is>
       </c>
       <c r="D98" s="2" t="n"/>
@@ -2414,17 +2414,17 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>A098</t>
+          <t>AN098</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>qhurukutu</t>
+          <t>jupha llamayu</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>tórtola</t>
+          <t>abril</t>
         </is>
       </c>
       <c r="D99" s="2" t="n"/>
@@ -2434,17 +2434,17 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>A099</t>
+          <t>AN099</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>laka</t>
+          <t>para</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>boca</t>
+          <t>frente</t>
         </is>
       </c>
       <c r="D100" s="2" t="n"/>
@@ -2454,17 +2454,17 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>A100</t>
+          <t>AN100</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>tawaqu</t>
+          <t>aka</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>la joven</t>
+          <t>esto, este, esta</t>
         </is>
       </c>
       <c r="D101" s="2" t="n"/>

</xml_diff>